<commit_message>
fix #45: fix opus template, propagate fill and formulas in table, fix link existence
</commit_message>
<xml_diff>
--- a/resources/xlsx_templates/opus.xlsx
+++ b/resources/xlsx_templates/opus.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbrandt/code/birddog/resources/xlsx_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53973DCC-1918-0B44-9C52-58588C3C4058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D1376F2-A92B-2C4E-BB23-303C9D5E4084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24360" yWindow="22640" windowWidth="31580" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="35160" yWindow="15160" windowWidth="34780" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="{shortname}" sheetId="4" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="55">
   <si>
     <t>source:</t>
   </si>
@@ -211,6 +211,12 @@
   </si>
   <si>
     <t>__EQ__COUNTA(H$__FIRST__:H__LAST__)-COUNTIF(H$__FIRST__:H__LAST__,"")</t>
+  </si>
+  <si>
+    <t>{col}=IF($F7="P1",CONCATENATE($A$1,"-",$G$1,"-",$H$1,"-",$A7),"")</t>
+  </si>
+  <si>
+    <t>{col}=IF($F7="P2",CONCATENATE($A$1,"-",$G$1,"-",$H$1,"-",$A7),"")</t>
   </si>
 </sst>
 </file>
@@ -1175,7 +1181,7 @@
         <v>24</v>
       </c>
       <c r="H7" s="59" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="I7" s="60" t="s">
         <v>24</v>
@@ -1183,8 +1189,8 @@
       <c r="J7" s="60" t="s">
         <v>24</v>
       </c>
-      <c r="K7" s="59" t="s">
-        <v>24</v>
+      <c r="K7" s="60" t="s">
+        <v>54</v>
       </c>
       <c r="L7" s="60" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
configurable download settings; breadcrumbs now use page lineage
</commit_message>
<xml_diff>
--- a/resources/xlsx_templates/opus.xlsx
+++ b/resources/xlsx_templates/opus.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbrandt/code/birddog/resources/xlsx_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F3FC5E3-D651-234F-AD37-0FB6578EBDEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5C5BCD4-F348-B04D-889A-F4909673E249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35160" yWindow="15160" windowWidth="34780" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="36000" windowHeight="22500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="{shortname}" sheetId="4" r:id="rId1"/>
+    <sheet name="{display_name}" sheetId="4" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>